<commit_message>
Sitemapa a feature breakdown sladene s wireframem
- sitemapa: pojmy, jak vznika a probiha trenink, vysvetleni nelinearity a vetveni, obrazovky podle Figmy, rozdily oproti upravenemu planu, otazky pro PO
- feature breakdown: pozvanku posila trener (F-08, F-09, F-11), cviky a sekvence (F-13), nova F-43 Pruchod treninkem, otevrene otazky z wireframu
- otazky-na-klienta: otazka 7 oznacena jako rozhodnuta

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018sH2sJcanJ9W5N2ME2yEuN
</commit_message>
<xml_diff>
--- a/docs/vystupy/feature-breakdown.xlsx
+++ b/docs/vystupy/feature-breakdown.xlsx
@@ -434,7 +434,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tým 5 · nástřel na hackathon 9. 10. 2026, vše ve stavu „Navrženo“ k projednání s PO. Řádky se zdrojem „Předpoklad týmu“ ověřit v rozhovoru. Priorita, Zdroj a Stav mají rozbalovací seznam.</t>
+          <t>Tým 5 · nástřel na hackathon 9. 10. 2026, sladěný s wireframem ve Figmě, vše ve stavu „Navrženo“ k projednání s PO. Čísla otázek v závorce odkazují na sitemapa.md, část Otázky pro PO. Priorita, Zdroj a Stav mají rozbalovací seznam.</t>
         </is>
       </c>
     </row>
@@ -523,7 +523,7 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Je trenér zvláštní typ účtu, nebo stačí role podle toho, čí je pes?</t>
+          <t>Rozhodnuto: trenér je placený účet a zve klienty. Může psovod aplikaci používat i bez trenéra? (otázka 6, 9)</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
@@ -811,17 +811,17 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Pozvání trenéra e-mailem</t>
+          <t>Trenér pozve klienta</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Psovod pošle trenérovi pozvánku, po přijetí trenér psa vidí. Nahrazuje screenshoty sešitu.</t>
+          <t>Trenér pošle klientovi pozvánku e-mailem nebo mu předá kód (třeba na lekci). Aplikaci platí trenér, proto zve on.</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Psovod</t>
+          <t>Trenér</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
@@ -831,12 +831,12 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
+          <t>Tým</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Co když pozvaný trenér ještě nemá účet?</t>
+          <t>Zve trenér člověka, nebo konkrétního psa? Co když klient už účet má? (otázka 7)</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
@@ -858,17 +858,17 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Připojení psa kódem</t>
+          <t>Přijetí pozvánky („Mám pozvánku“)</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Psovod ukáže kód (třeba na lekci), trenér ho zadá a psa si připojí.</t>
+          <t>Klient na úvodní obrazovce zvolí „Mám pozvánku“, zadá kód nebo otevře odkaz, zaregistruje se a propojí se s trenérem.</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Psovod, trenér</t>
+          <t>Psovod</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
@@ -878,12 +878,12 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Klient</t>
+          <t>Tým</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>Jak dlouho kód platí?</t>
+          <t>Jak dlouho kód platí? (otázka 7)</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
@@ -910,12 +910,12 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Psovod ukončí spolupráci a trenér psa přestane vidět.</t>
+          <t>Trenér nebo psovod ukončí spolupráci, trenér psa přestane vidět.</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Psovod</t>
+          <t>Psovod, trenér</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -948,17 +948,17 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Trenér pozve klienta</t>
+          <t>Psovod pozve trenéra</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Trenér pošle klientovi výzvu, ať mu psa nasdílí. Usnadní trenérovi převést klienty z WhatsAppu.</t>
+          <t>Obrácený směr: psovod, který už trenéra má, ho pozve do aplikace.</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Trenér</t>
+          <t>Psovod</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
@@ -971,7 +971,7 @@
           <t>Předpoklad týmu</t>
         </is>
       </c>
-      <c r="H15" s="5" t="n"/>
+      <c r="H15" s="5" t="inlineStr"/>
       <c r="I15" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>Má cíl termín nebo měřitelné kritérium splnění?</t>
+          <t>Ve wireframu cíle nejsou. Plánuje trenér vždy k cíli, nebo stačí trénink pro psa s disciplínou? (otázka 2)</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
@@ -1038,12 +1038,12 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Úkoly k cíli</t>
+          <t>Cviky a sekvence cviků</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>K cíli se zapíší dílčí úkoly v pořadí (oční kontakt → delší podržení → rušivky). Kdykoli jde úkol přidat, upravit nebo vložit mezikrok.</t>
+          <t>Plán se skládá z bloků „Jednotlivý cvik“ (např. Běh v plném tahu 400 m) a „Sekvence cviků“ (několik cviků vždy po sobě). Blok jde přidat (+), upravit, smazat (koš) nebo vložit jako mezikrok.</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>Posouvá se na další úkol jen ručně, nebo i podle % úspěšnosti?</t>
+          <t>Posouvá se jen ručně, nebo i podle % úspěšnosti? (otázka 1 v otazky-na-klienta.md)</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
@@ -1133,7 +1133,7 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Cíl se rozdělí na dvě cesty, které se trénují souběžně.</t>
+          <t>Cesta se rozdělí na dvě větve, které se trénují souběžně, a později se mohou znovu spojit (tak to kreslí wireframe).</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -1153,7 +1153,7 @@
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>Jak vypadá větvení na konkrétním příkladu se Zoe? Cesty se zase spojí?</t>
+          <t>Větví se plán k cíli v čase, nebo jeden trénink? Trénují se obě větve, nebo se jedna vybere? Příklad se Zoe. (otázka 1)</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
@@ -1175,12 +1175,12 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Úpravy plánu trenérem</t>
+          <t>Tvorba a úpravy plánu trenérem</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Přizvaný trenér zakládá a upravuje cíle a úkoly stejně jako psovod.</t>
+          <t>Trenér skládá a upravuje plán psa klienta na obrazovce „Tvorba tréninku“.</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -1198,7 +1198,11 @@
           <t>Klient</t>
         </is>
       </c>
-      <c r="H20" s="5" t="n"/>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>Smí plán upravovat i psovod, jak říká upravený plán? (otázka 6)</t>
+        </is>
+      </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
@@ -1309,7 +1313,7 @@
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Hlavní obrazovka: aktuální týden po dnech, úkoly ze všech disciplín najednou.</t>
+          <t>Aktuální týden po dnech, tréninky všech psů najednou, barevně podle psa. Po kliknutí na den karta tréninku se seznamem cviků.</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -1327,7 +1331,11 @@
           <t>Klient</t>
         </is>
       </c>
-      <c r="H23" s="5" t="n"/>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>Barva podle psa (wireframe), nebo podle disciplíny?</t>
+        </is>
+      </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
@@ -1372,7 +1380,7 @@
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>Cvičí se jeden úkol v týdnu opakovaně (např. 3× pozornost)?</t>
+          <t>Rozvrhne aplikace cviky z plánu do dnů sama („vygenerovaný popis“ ve wireframu), nebo se trénink zařadí ručně? Opakuje se úkol v týdnu? (otázka 5)</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
@@ -1532,7 +1540,7 @@
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Po tréninku psovod zapíše % úspěšnosti a poznámku — rychle, z mobilu, přímo z týdne.</t>
+          <t>Po tréninku psovod na obrazovce „Konec“ zapíše výsledek a komentář — rychle, z mobilu.</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -1552,7 +1560,7 @@
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>Jak se % určuje (počet úspěšných opakování, odhad)?</t>
+          <t>Ve wireframu % chybí. Zadává se % za každý cvik, za celý trénink, nebo vůbec? (otázka 3)</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
@@ -1597,7 +1605,11 @@
           <t>Klient</t>
         </is>
       </c>
-      <c r="H29" s="5" t="n"/>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>Wireframe má „Nahrát video“, upravený plán upload vylučuje (F-28). V MVP vložit odkaz? (otázka 4)</t>
+        </is>
+      </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
@@ -1622,7 +1634,7 @@
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>U úkolu jsou všechny záznamy v čase, jde porovnat, co fungovalo.</t>
+          <t>Na detailu psa jsou „Aktivity“: odcvičené tréninky po dnech se záznamy, jde porovnat, co fungovalo.</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -1789,12 +1801,12 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Komentáře pod úkolem</t>
+          <t>Komentáře k tréninku</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Psovod a trenér si pod konkrétním úkolem píšou, trenér reaguje na video a výsledek. Nahrazuje WhatsApp.</t>
+          <t>Psovod pošle k tréninku komentář, trenér mu odpoví ve vlákně a reaguje na video a výsledek. Nahrazuje WhatsApp.</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -1812,7 +1824,11 @@
           <t>Klient</t>
         </is>
       </c>
-      <c r="H34" s="5" t="n"/>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>Wireframe má jen komentář psovoda. Kde trenér odpoví a kde psovod odpověď uvidí? (otázka 8)</t>
+        </is>
+      </c>
       <c r="I34" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
@@ -1837,7 +1853,7 @@
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Trenér vidí všechny psy, které mu klienti nasdíleli, a otevře jejich týden a plán.</t>
+          <t>Trenér vidí své klienty (jméno, e-mail) a přes ně jejich psy, týden a plán.</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -1880,7 +1896,7 @@
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Trenér vidí nové záznamy od klientů, na které ještě nereagoval.</t>
+          <t>U klienta svítí štítek „čeká na reakci“, dokud trenér nezareaguje na jeho nové záznamy.</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -1895,7 +1911,7 @@
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>Předpoklad týmu</t>
+          <t>Tým</t>
         </is>
       </c>
       <c r="H36" s="5" t="n"/>
@@ -2348,15 +2364,51 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="5" t="n"/>
-      <c r="B47" s="5" t="n"/>
-      <c r="C47" s="5" t="n"/>
-      <c r="D47" s="5" t="n"/>
-      <c r="E47" s="5" t="n"/>
-      <c r="F47" s="5" t="n"/>
-      <c r="G47" s="5" t="n"/>
-      <c r="H47" s="5" t="n"/>
-      <c r="I47" s="5" t="n"/>
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>F-43</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Záznam tréninku</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>Průchod tréninkem</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Psovod otevře dnešní trénink a prochází cviky jeden po druhém („Aktuální cvik 3/20“), na konci přejde na zápis výsledku.</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Psovod</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>Tým</t>
+        </is>
+      </c>
+      <c r="H47" s="5" t="inlineStr">
+        <is>
+          <t>Znamenají šipky další cvik v dnešním tréninku, nebo posun v plánu (F-14)?</t>
+        </is>
+      </c>
+      <c r="I47" s="5" t="inlineStr">
+        <is>
+          <t>Navrženo</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="n"/>
@@ -2638,7 +2690,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Psovod a trenér se propojí nad konkrétním psem.</t>
+          <t>Trenér pozve klienta a propojí se s jeho psem.</t>
         </is>
       </c>
       <c r="C7" s="5">

</xml_diff>

<commit_message>
Sitemapa a breakdown uz neodkazuji na upraveny plan, srovnani s feature breakdownem
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018sH2sJcanJ9W5N2ME2yEuN
</commit_message>
<xml_diff>
--- a/docs/vystupy/feature-breakdown.xlsx
+++ b/docs/vystupy/feature-breakdown.xlsx
@@ -1200,7 +1200,7 @@
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>Smí plán upravovat i psovod, jak říká upravený plán? (otázka 6)</t>
+          <t>Smí plán upravovat i psovod? Wireframe počítá jen s trenérem. (otázka 6)</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
@@ -1607,7 +1607,7 @@
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>Wireframe má „Nahrát video“, upravený plán upload vylučuje (F-28). V MVP vložit odkaz? (otázka 4)</t>
+          <t>Wireframe má „Nahrát video“, nahrávání na náš server je mimo rozsah (F-28). V MVP vložit odkaz? (otázka 4)</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Feature breakdown a sitemapa srovnane podle wireframu
- plan sklada trener, bez samostatnych cilu (epic Plan treninku)
- po treninku video a komentar, % a forma videa jako otazky pro PO
- odstranena sekce s rozdily, otazky preformulovane

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018sH2sJcanJ9W5N2ME2yEuN
</commit_message>
<xml_diff>
--- a/docs/vystupy/feature-breakdown.xlsx
+++ b/docs/vystupy/feature-breakdown.xlsx
@@ -503,7 +503,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Psovod i trenér si založí účet e-mailem a heslem. Bez účtu nejde psa sdílet.</t>
+          <t>Psovod i trenér si založí účet e-mailem a heslem. Bez účtu se klient s trenérem nepropojí.</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -636,7 +636,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Psovod založí psa (jméno, plemeno). Pes je středem plánu, rozvrhu i sdílení.</t>
+          <t>Psovod založí psa (jméno, plemeno, fotka). Pes je středem plánu, kalendáře i spolupráce s trenérem.</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -986,22 +986,22 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Cíle a plán</t>
+          <t>Plán tréninku</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Cíl v disciplíně</t>
+          <t>Plán tréninku pro psa</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Psovod nebo trenér založí cíl, např. „5 km pod 5 min/km“.</t>
+          <t>Trenér založí pro psa klienta plán v disciplíně, např. „Trénink pro Rexe“ (obrazovka Tvorba tréninku).</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Psovod, trenér</t>
+          <t>Trenér</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -1016,7 +1016,7 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>Ve wireframu cíle nejsou. Plánuje trenér vždy k cíli, nebo stačí trénink pro psa s disciplínou? (otázka 2)</t>
+          <t>Chcete u plánu i cíl (např. 5 km pod 5 min/km)? (otázka 2)</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Cíle a plán</t>
+          <t>Plán tréninku</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Psovod, trenér</t>
+          <t>Trenér</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Cíle a plán</t>
+          <t>Plán tréninku</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -1086,12 +1086,12 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Je vidět, na kterém úkolu pes je. Když nejde, vrátí se o krok; když to umí, úkol se přeskočí.</t>
+          <t>Je vidět, na kterém cviku pes je. Když nejde, vrátí se o krok; když to umí, cvik se přeskočí.</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Psovod, trenér</t>
+          <t>Trenér</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
@@ -1123,7 +1123,7 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Cíle a plán</t>
+          <t>Plán tréninku</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Psovod, trenér</t>
+          <t>Trenér</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
@@ -1153,7 +1153,7 @@
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>Větví se plán k cíli v čase, nebo jeden trénink? Trénují se obě větve, nebo se jedna vybere? Příklad se Zoe. (otázka 1)</t>
+          <t>Větví se plán na několik týdnů, nebo jeden trénink? Trénují se obě větve, nebo se jedna vybere? Příklad se Zoe. (otázka 1)</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
@@ -1170,17 +1170,17 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Cíle a plán</t>
+          <t>Plán tréninku</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Tvorba a úpravy plánu trenérem</t>
+          <t>Úpravy plánu podle výsledků</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Trenér skládá a upravuje plán psa klienta na obrazovce „Tvorba tréninku“.</t>
+          <t>Trenér po reakci na odeslaný trénink upraví plán v Tvorbě tréninku.</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>Smí plán upravovat i psovod? Wireframe počítá jen s trenérem. (otázka 6)</t>
+          <t>Má plán upravovat i psovod? (otázka 6)</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
@@ -1217,22 +1217,22 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Cíle a plán</t>
+          <t>Plán tréninku</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Dokončení a archiv cíle</t>
+          <t>Dokončení a archiv plánu</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Splněný nebo opuštěný cíl zmizí z aktivních, ale zůstane v historii.</t>
+          <t>Dokončený nebo opuštěný plán zmizí z aktivních, ale zůstane v historii.</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>Psovod, trenér</t>
+          <t>Trenér</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
@@ -1260,12 +1260,12 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Cíle a plán</t>
+          <t>Plán tréninku</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Kopie cíle / šablona trenéra</t>
+          <t>Kopie plánu / šablona trenéra</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -1331,11 +1331,7 @@
           <t>Klient</t>
         </is>
       </c>
-      <c r="H23" s="5" t="inlineStr">
-        <is>
-          <t>Barva podle psa (wireframe), nebo podle disciplíny?</t>
-        </is>
-      </c>
+      <c r="H23" s="5" t="n"/>
       <c r="I23" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
@@ -1355,12 +1351,12 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Naplánování úkolu na den</t>
+          <t>Naplánování tréninku na den</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Aktivní úkol z libovolného cíle se zařadí do konkrétního dne.</t>
+          <t>Trénink z plánu se zařadí do konkrétního dne.</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -1380,7 +1376,7 @@
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>Rozvrhne aplikace cviky z plánu do dnů sama („vygenerovaný popis“ ve wireframu), nebo se trénink zařadí ručně? Opakuje se úkol v týdnu? (otázka 5)</t>
+          <t>Rozvrhne aplikace cviky z plánu do dnů sama („vygenerovaný popis“ ve wireframu), nebo se trénink zařadí ručně? Může být stejný trénink v týdnu vícekrát? (otázka 5)</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
@@ -1535,12 +1531,12 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Zápis výsledku</t>
+          <t>Odeslání tréninku</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Po tréninku psovod na obrazovce „Konec“ zapíše výsledek a komentář — rychle, z mobilu.</t>
+          <t>Na obrazovce „Konec“ psovod napíše komentář a odešle trénink trenérovi — rychle, z mobilu.</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -1560,7 +1556,7 @@
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>Ve wireframu % chybí. Zadává se % za každý cvik, za celý trénink, nebo vůbec? (otázka 3)</t>
+          <t>Má psovod zadávat i % úspěšnosti? Za každý cvik, nebo za celý trénink? (otázka 3)</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
@@ -1582,12 +1578,12 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Odkaz na video</t>
+          <t>Video z tréninku</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>K záznamu se přiloží odkaz (YouTube unlisted, cloud), video už neleží odpojené v galerii.</t>
+          <t>Na obrazovce „Konec“ psovod tlačítkem „Nahrát video“ přiloží video z tréninku, takže už neleží odpojené v galerii.</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -1607,7 +1603,7 @@
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>Wireframe má „Nahrát video“, nahrávání na náš server je mimo rozsah (F-28). V MVP vložit odkaz? (otázka 4)</t>
+          <t>Stačí v MVP odkaz (YouTube, Disk), nebo nahrání souboru (F-28)? (otázka 4)</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
@@ -1629,7 +1625,7 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Historie tréninků úkolu</t>
+          <t>Historie tréninků psa</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
@@ -1677,7 +1673,7 @@
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Vývoj % v čase u úkolu nebo cíle.</t>
+          <t>Vývoj % v čase u psa nebo plánu.</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -1695,7 +1691,11 @@
           <t>Předpoklad týmu</t>
         </is>
       </c>
-      <c r="H31" s="5" t="n"/>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>Jen pokud se bude zadávat % úspěšnosti (otázka 3).</t>
+        </is>
+      </c>
       <c r="I31" s="5" t="inlineStr">
         <is>
           <t>Navrženo</t>
@@ -1720,7 +1720,7 @@
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Řeší se externími odkazy.</t>
+          <t>Vlastní úložiště videí je drahé, v MVP ho nestavíme (viz F-25, otázka 4).</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -1806,7 +1806,7 @@
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Psovod pošle k tréninku komentář, trenér mu odpoví ve vlákně a reaguje na video a výsledek. Nahrazuje WhatsApp.</t>
+          <t>Psovod pošle s tréninkem komentář, trenér mu odpoví ve vlákně a reaguje na video. Nahrazuje WhatsApp.</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>Wireframe má jen komentář psovoda. Kde trenér odpoví a kde psovod odpověď uvidí? (otázka 8)</t>
+          <t>Kde psovod odpověď trenéra uvidí? (otázka 8)</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr">
@@ -2381,7 +2381,7 @@
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>Psovod otevře dnešní trénink a prochází cviky jeden po druhém („Aktuální cvik 3/20“), na konci přejde na zápis výsledku.</t>
+          <t>Psovod otevře dnešní trénink a prochází cviky jeden po druhém („Aktuální cvik 3/20“), na konci přejde na obrazovku „Konec“.</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -2710,12 +2710,12 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Cíle a plán</t>
+          <t>Plán tréninku</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Nelineární plán: cíl → úkoly, návrat, přeskočení, větvení.</t>
+          <t>Trenér skládá plán z cviků a sekvencí, s návratem, přeskočením a větvením.</t>
         </is>
       </c>
       <c r="C8" s="5">
@@ -2740,7 +2740,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Jedna obrazovka s týdnem napříč všemi disciplínami.</t>
+          <t>Kalendář s tréninky všech psů na celý týden.</t>
         </is>
       </c>
       <c r="C9" s="5">
@@ -2765,7 +2765,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Po tréninku zapsat % úspěšnosti, poznámku a video.</t>
+          <t>Psovod projde trénink a odešle video a komentář.</t>
         </is>
       </c>
       <c r="C10" s="5">

</xml_diff>

<commit_message>
Sitemapa: jak trener zada klientovi trenink
- cesta Klienti -> Detail klienta -> Pes -> Tvorba treninku -> Naplanovat trenink
- nova obrazovka Naplanovat trenink (chybi ve wireframu), F-20 ji popisuje
- odstranena poznamka Rozhodnuto

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018sH2sJcanJ9W5N2ME2yEuN
</commit_message>
<xml_diff>
--- a/docs/vystupy/feature-breakdown.xlsx
+++ b/docs/vystupy/feature-breakdown.xlsx
@@ -1356,12 +1356,12 @@
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Trénink z plánu se zařadí do konkrétního dne.</t>
+          <t>Trenér po uložení tréninku vybere dny v týdnu a období (od–do). Trénink se objeví klientovi v Týdnu.</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Psovod</t>
+          <t>Trenér</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
@@ -1376,7 +1376,7 @@
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>Rozvrhne aplikace cviky z plánu do dnů sama („vygenerovaný popis“ ve wireframu), nebo se trénink zařadí ručně? Může být stejný trénink v týdnu vícekrát? (otázka 5)</t>
+          <t>Vybere dny trenér, nebo má aplikace trénink rozvrhnout sama („vygenerovaný popis“ ve wireframu)? (otázka 5)</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Otazky pro PO jen v otazky-na-klienta.md
- doplneny podotazky z wireframu k otazkam 1, 2, 3, 5, 6, 8, 9
- nove otazky 4 (cil u planu) a 10 (navigace podle role), ostatni precislovany
- sitemapa odkazuje na otazky-na-klienta, breakdown na nove cislovani

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018sH2sJcanJ9W5N2ME2yEuN
</commit_message>
<xml_diff>
--- a/docs/vystupy/feature-breakdown.xlsx
+++ b/docs/vystupy/feature-breakdown.xlsx
@@ -434,7 +434,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tým 5 · nástřel na hackathon 9. 10. 2026, sladěný s wireframem ve Figmě, vše ve stavu „Navrženo“ k projednání s PO. Čísla otázek v závorce odkazují na sitemapa.md, část Otázky pro PO. Priorita, Zdroj a Stav mají rozbalovací seznam.</t>
+          <t>Tým 5 · nástřel na hackathon 9. 10. 2026, sladěný s wireframem ve Figmě, vše ve stavu „Navrženo“ k projednání s PO. Čísla otázek v závorce odkazují na otazky-na-klienta.md. Priorita, Zdroj a Stav mají rozbalovací seznam.</t>
         </is>
       </c>
     </row>
@@ -523,7 +523,7 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Rozhodnuto: trenér je placený účet a zve klienty. Může psovod aplikaci používat i bez trenéra? (otázka 6, 9)</t>
+          <t>Rozhodnuto: trenér je placený účet a zve klienty. Může psovod aplikaci používat i bez trenéra? (otázka 2, 10)</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Zve trenér člověka, nebo konkrétního psa? Co když klient už účet má? (otázka 7)</t>
+          <t>Zve trenér člověka, nebo konkrétního psa? Co když klient už účet má? (otázka 8)</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
@@ -883,7 +883,7 @@
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>Jak dlouho kód platí? (otázka 7)</t>
+          <t>Jak dlouho kód platí? (otázka 8)</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
@@ -1016,7 +1016,7 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>Chcete u plánu i cíl (např. 5 km pod 5 min/km)? (otázka 2)</t>
+          <t>Chcete u plánu i cíl (např. 5 km pod 5 min/km)? (otázka 4)</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>Posouvá se jen ručně, nebo i podle % úspěšnosti? (otázka 1 v otazky-na-klienta.md)</t>
+          <t>Posouvá se jen ručně, nebo i podle % úspěšnosti? (otázka 1)</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>Má plán upravovat i psovod? (otázka 6)</t>
+          <t>Má plán upravovat i psovod? (otázka 2)</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>Stačí v MVP odkaz (YouTube, Disk), nebo nahrání souboru (F-28)? (otázka 4)</t>
+          <t>Stačí v MVP odkaz (YouTube, Disk), nebo nahrání souboru (F-28)? (otázka 6)</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>Kde psovod odpověď trenéra uvidí? (otázka 8)</t>
+          <t>Kde psovod odpověď trenéra uvidí? (otázka 9)</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr">

</xml_diff>